<commit_message>
KT progress: 1 topic updated by Akshay
</commit_message>
<xml_diff>
--- a/coveo-kt-tracker.xlsx
+++ b/coveo-kt-tracker.xlsx
@@ -5,7 +5,8 @@
   <sheets>
     <sheet name="Roadmap" sheetId="1" r:id="rId1"/>
     <sheet name="How to use" sheetId="2" r:id="rId2"/>
-    <sheet name="People" sheetId="3" r:id="rId3"/>
+    <sheet name="Questions" sheetId="3" r:id="rId3"/>
+    <sheet name="People" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -488,7 +489,7 @@
         <v/>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>1 open of 1</v>
       </c>
     </row>
     <row r="3">
@@ -3540,7 +3541,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
@@ -3572,27 +3573,98 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Topic is the identity of a row. Renaming one restarts its progress.</v>
+        <v>The Questions sheet holds one row per message: a Question row, then its Comment rows, grouped by Topic and Thread.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Commit this file over the old one in the repository to publish progress.</v>
+        <v>Topic is the identity of a row. Renaming one restarts its progress.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Commit this file over the old one in the repository to publish progress.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>Do not put organization IDs, source IDs, endpoints, key names or key values in this file.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G2"/>
+  <cols>
+    <col min="1" max="1" width="44.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="9.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Topic</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Thread</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Kind</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Text</v>
+      </c>
+      <c r="E1" t="str">
+        <v>By</v>
+      </c>
+      <c r="F1" t="str">
+        <v>On</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>What Coveo is and where it fits in our stack</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Question</v>
+      </c>
+      <c r="D2" t="str">
+        <v>what</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Divyashree</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Sep 15</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Open</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <cols>

</xml_diff>

<commit_message>
KT progress: topic list edited by AKSHAY
</commit_message>
<xml_diff>
--- a/coveo-kt-tracker.xlsx
+++ b/coveo-kt-tracker.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L81"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="40.83203125" customWidth="1"/>
@@ -653,19 +653,19 @@
         <v/>
       </c>
       <c r="C7" t="str">
-        <v>Prod and non-prod pairing for each licence</v>
+        <v>What each licence limits in practice</v>
       </c>
       <c r="D7" t="str">
-        <v>Which non-prod organization belongs to which prod organization, naming convention, and how access is requested for each.</v>
+        <v>Index size, source count, query volume, number of ML models. Where to read current consumption in the console.</v>
       </c>
       <c r="E7" t="str">
-        <v>Demo</v>
+        <v>Concept</v>
       </c>
       <c r="F7" t="str">
-        <v>Internal - environment matrix</v>
+        <v>docs.coveo.com - search: licence limits</v>
       </c>
       <c r="G7" t="str">
-        <v/>
+        <v>Contractual figures come from the contract, not from the docs.</v>
       </c>
       <c r="H7" t="str">
         <v>No</v>
@@ -685,25 +685,25 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>1. Coveo Platform overview</v>
+        <v>2. Platform foundation and the Admin Console</v>
       </c>
       <c r="B8" t="str">
-        <v/>
+        <v>Find anything in the Administration Console without help, and know what each tab changes.</v>
       </c>
       <c r="C8" t="str">
-        <v>What each licence limits in practice</v>
+        <v>Moving configuration between organizations</v>
       </c>
       <c r="D8" t="str">
-        <v>Index size, source count, query volume, number of ML models. Where to read current consumption in the console.</v>
+        <v>What is configured per organization, what we keep identical across prod and non-prod, and how a change is promoted.</v>
       </c>
       <c r="E8" t="str">
         <v>Concept</v>
       </c>
       <c r="F8" t="str">
-        <v>docs.coveo.com - search: licence limits</v>
+        <v>docs.coveo.com - search: resource snapshots</v>
       </c>
       <c r="G8" t="str">
-        <v>Contractual figures come from the contract, not from the docs.</v>
+        <v/>
       </c>
       <c r="H8" t="str">
         <v>No</v>
@@ -726,19 +726,19 @@
         <v>2. Platform foundation and the Admin Console</v>
       </c>
       <c r="B9" t="str">
-        <v>Find anything in the Administration Console without help, and know what each tab changes.</v>
+        <v/>
       </c>
       <c r="C9" t="str">
-        <v>Moving configuration between organizations</v>
+        <v>Content tab: sources and Content Browser</v>
       </c>
       <c r="D9" t="str">
-        <v>What is configured per organization, what we keep identical across prod and non-prod, and how a change is promoted.</v>
+        <v>Source list and status, adding and editing a source, inspecting an indexed item and its fields.</v>
       </c>
       <c r="E9" t="str">
-        <v>Concept</v>
+        <v>Demo</v>
       </c>
       <c r="F9" t="str">
-        <v>docs.coveo.com - search: resource snapshots</v>
+        <v>docs.coveo.com - search: Content Browser</v>
       </c>
       <c r="G9" t="str">
         <v/>
@@ -767,16 +767,16 @@
         <v/>
       </c>
       <c r="C10" t="str">
-        <v>Content tab: sources and Content Browser</v>
+        <v>Content tab: fields and mappings</v>
       </c>
       <c r="D10" t="str">
-        <v>Source list and status, adding and editing a source, inspecting an indexed item and its fields.</v>
+        <v>Field list, field types, facet, sortable and free-text options, and where mappings are defined per source.</v>
       </c>
       <c r="E10" t="str">
         <v>Demo</v>
       </c>
       <c r="F10" t="str">
-        <v>docs.coveo.com - search: Content Browser</v>
+        <v>docs.coveo.com - search: fields</v>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -805,16 +805,16 @@
         <v/>
       </c>
       <c r="C11" t="str">
-        <v>Content tab: fields and mappings</v>
+        <v>Content tab: security identities and providers</v>
       </c>
       <c r="D11" t="str">
-        <v>Field list, field types, facet, sortable and free-text options, and where mappings are defined per source.</v>
+        <v>Which of our content is secured, which is public, and how identities reach the index.</v>
       </c>
       <c r="E11" t="str">
-        <v>Demo</v>
+        <v>Concept</v>
       </c>
       <c r="F11" t="str">
-        <v>docs.coveo.com - search: fields</v>
+        <v>docs.coveo.com - search: security identities</v>
       </c>
       <c r="G11" t="str">
         <v/>
@@ -843,16 +843,16 @@
         <v/>
       </c>
       <c r="C12" t="str">
-        <v>Content tab: security identities and providers</v>
+        <v>Search Optimization tab: query pipelines and statements</v>
       </c>
       <c r="D12" t="str">
-        <v>Which of our content is secured, which is public, and how identities reach the index.</v>
+        <v>Pipeline list, routing conditions, statement types, and which pipeline serves which storefront.</v>
       </c>
       <c r="E12" t="str">
-        <v>Concept</v>
+        <v>Demo</v>
       </c>
       <c r="F12" t="str">
-        <v>docs.coveo.com - search: security identities</v>
+        <v>docs.coveo.com - search: query pipelines</v>
       </c>
       <c r="G12" t="str">
         <v/>
@@ -881,16 +881,16 @@
         <v/>
       </c>
       <c r="C13" t="str">
-        <v>Search Optimization tab: query pipelines and statements</v>
+        <v>Machine Learning tab</v>
       </c>
       <c r="D13" t="str">
-        <v>Pipeline list, routing conditions, statement types, and which pipeline serves which storefront.</v>
+        <v>Model list, status, associations to pipelines, and what the model detail page tells you.</v>
       </c>
       <c r="E13" t="str">
         <v>Demo</v>
       </c>
       <c r="F13" t="str">
-        <v>docs.coveo.com - search: query pipelines</v>
+        <v>docs.coveo.com - search: Coveo Machine Learning</v>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -919,16 +919,16 @@
         <v/>
       </c>
       <c r="C14" t="str">
-        <v>Machine Learning tab</v>
+        <v>Analytics tab: dashboards, reports and visit inspection</v>
       </c>
       <c r="D14" t="str">
-        <v>Model list, status, associations to pipelines, and what the model detail page tells you.</v>
+        <v>The dashboards we actually use, how to build a report, and how to open a single visit.</v>
       </c>
       <c r="E14" t="str">
         <v>Demo</v>
       </c>
       <c r="F14" t="str">
-        <v>docs.coveo.com - search: Coveo Machine Learning</v>
+        <v>docs.coveo.com - search: usage analytics dashboards</v>
       </c>
       <c r="G14" t="str">
         <v/>
@@ -957,16 +957,16 @@
         <v/>
       </c>
       <c r="C15" t="str">
-        <v>Analytics tab: dashboards, reports and visit inspection</v>
+        <v>Commerce tab: catalogs, product listings, Merchandising Hub</v>
       </c>
       <c r="D15" t="str">
-        <v>The dashboards we actually use, how to build a report, and how to open a single visit.</v>
+        <v>How a catalog is configured, what a product listing is, and where merchandising rules live.</v>
       </c>
       <c r="E15" t="str">
         <v>Demo</v>
       </c>
       <c r="F15" t="str">
-        <v>docs.coveo.com - search: usage analytics dashboards</v>
+        <v>docs.coveo.com - search: catalog product listing</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -995,19 +995,19 @@
         <v/>
       </c>
       <c r="C16" t="str">
-        <v>Commerce tab: catalogs, product listings, Merchandising Hub</v>
+        <v>Organization tab: members, groups and API keys</v>
       </c>
       <c r="D16" t="str">
-        <v>How a catalog is configured, what a product listing is, and where merchandising rules live.</v>
+        <v>Group privileges, creating and scoping an API key, and reading the activity log.</v>
       </c>
       <c r="E16" t="str">
-        <v>Demo</v>
+        <v>Hands-on</v>
       </c>
       <c r="F16" t="str">
-        <v>docs.coveo.com - search: catalog product listing</v>
+        <v>docs.coveo.com - search: API key privileges</v>
       </c>
       <c r="G16" t="str">
-        <v/>
+        <v>Never share key values. Grant through groups.</v>
       </c>
       <c r="H16" t="str">
         <v>No</v>
@@ -1033,19 +1033,19 @@
         <v/>
       </c>
       <c r="C17" t="str">
-        <v>Organization tab: members, groups and API keys</v>
+        <v>Organization tab: settings, licence and consumption</v>
       </c>
       <c r="D17" t="str">
-        <v>Group privileges, creating and scoping an API key, and reading the activity log.</v>
+        <v>Organization settings we must not change casually, and where licence usage is reported.</v>
       </c>
       <c r="E17" t="str">
-        <v>Hands-on</v>
+        <v>Demo</v>
       </c>
       <c r="F17" t="str">
-        <v>docs.coveo.com - search: API key privileges</v>
+        <v>docs.coveo.com - search: organization settings</v>
       </c>
       <c r="G17" t="str">
-        <v>Never share key values. Grant through groups.</v>
+        <v/>
       </c>
       <c r="H17" t="str">
         <v>No</v>
@@ -1071,16 +1071,16 @@
         <v/>
       </c>
       <c r="C18" t="str">
-        <v>Organization tab: settings, licence and consumption</v>
+        <v>Quotas, limits and what happens at the ceiling</v>
       </c>
       <c r="D18" t="str">
-        <v>Organization settings we must not change casually, and where licence usage is reported.</v>
+        <v>Index and query limits, payload and rate limits, and the symptoms when one is hit.</v>
       </c>
       <c r="E18" t="str">
-        <v>Demo</v>
+        <v>Concept</v>
       </c>
       <c r="F18" t="str">
-        <v>docs.coveo.com - search: organization settings</v>
+        <v>docs.coveo.com - search: platform limits</v>
       </c>
       <c r="G18" t="str">
         <v/>
@@ -1109,16 +1109,16 @@
         <v/>
       </c>
       <c r="C19" t="str">
-        <v>Quotas, limits and what happens at the ceiling</v>
+        <v>Who owns what, and what needs approval</v>
       </c>
       <c r="D19" t="str">
-        <v>Index and query limits, payload and rate limits, and the symptoms when one is hit.</v>
+        <v>Which areas we change freely, which need a review, and which belong to the business.</v>
       </c>
       <c r="E19" t="str">
         <v>Concept</v>
       </c>
       <c r="F19" t="str">
-        <v>docs.coveo.com - search: platform limits</v>
+        <v>Internal - ways of working</v>
       </c>
       <c r="G19" t="str">
         <v/>
@@ -1141,22 +1141,22 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2. Platform foundation and the Admin Console</v>
+        <v>3. Dashboard configuration to the indexing JAR</v>
       </c>
       <c r="B20" t="str">
-        <v/>
+        <v>Trace every piece of console configuration and every key that the indexing JAR depends on.</v>
       </c>
       <c r="C20" t="str">
-        <v>Who owns what, and what needs approval</v>
+        <v>Which console configuration the JAR depends on</v>
       </c>
       <c r="D20" t="str">
-        <v>Which areas we change freely, which need a review, and which belong to the business.</v>
+        <v>The source it pushes to, the fields and mappings it assumes exist, and what breaks if any of them changes.</v>
       </c>
       <c r="E20" t="str">
         <v>Concept</v>
       </c>
       <c r="F20" t="str">
-        <v>Internal - ways of working</v>
+        <v>docs.coveo.com - search: push source</v>
       </c>
       <c r="G20" t="str">
         <v/>
@@ -1182,19 +1182,19 @@
         <v>3. Dashboard configuration to the indexing JAR</v>
       </c>
       <c r="B21" t="str">
-        <v>Trace every piece of console configuration and every key that the indexing JAR depends on.</v>
+        <v/>
       </c>
       <c r="C21" t="str">
-        <v>Which console configuration the JAR depends on</v>
+        <v>API keys the JAR uses and their privileges</v>
       </c>
       <c r="D21" t="str">
-        <v>The source it pushes to, the fields and mappings it assumes exist, and what breaks if any of them changes.</v>
+        <v>Minimum privileges for pushing content, one key per environment, and why an admin key is never used.</v>
       </c>
       <c r="E21" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F21" t="str">
-        <v>docs.coveo.com - search: push source</v>
+        <v>docs.coveo.com - search: API key privileges</v>
       </c>
       <c r="G21" t="str">
         <v/>
@@ -1223,19 +1223,19 @@
         <v/>
       </c>
       <c r="C22" t="str">
-        <v>API keys the JAR uses and their privileges</v>
+        <v>Where credentials live and how they rotate</v>
       </c>
       <c r="D22" t="str">
-        <v>Minimum privileges for pushing content, one key per environment, and why an admin key is never used.</v>
+        <v>The secret store or pipeline variables we use, rotation process, and the check that no key sits in the repo.</v>
       </c>
       <c r="E22" t="str">
-        <v>Hands-on</v>
+        <v>Concept</v>
       </c>
       <c r="F22" t="str">
-        <v>docs.coveo.com - search: API key privileges</v>
+        <v>Internal - secret management</v>
       </c>
       <c r="G22" t="str">
-        <v/>
+        <v>Rotate immediately if a key ever appears in a commit or a log.</v>
       </c>
       <c r="H22" t="str">
         <v>No</v>
@@ -1261,19 +1261,19 @@
         <v/>
       </c>
       <c r="C23" t="str">
-        <v>Where credentials live and how they rotate</v>
+        <v>The JAR configuration file, field by field</v>
       </c>
       <c r="D23" t="str">
-        <v>The secret store or pipeline variables we use, rotation process, and the check that no key sits in the repo.</v>
+        <v>Organization, source, region and endpoint settings, batch sizes, timeouts and retry values.</v>
       </c>
       <c r="E23" t="str">
-        <v>Concept</v>
+        <v>Code walkthrough</v>
       </c>
       <c r="F23" t="str">
-        <v>Internal - secret management</v>
+        <v>Internal - config reference</v>
       </c>
       <c r="G23" t="str">
-        <v>Rotate immediately if a key ever appears in a commit or a log.</v>
+        <v/>
       </c>
       <c r="H23" t="str">
         <v>No</v>
@@ -1299,10 +1299,10 @@
         <v/>
       </c>
       <c r="C24" t="str">
-        <v>The JAR configuration file, field by field</v>
+        <v>Configuration per environment and per store</v>
       </c>
       <c r="D24" t="str">
-        <v>Organization, source, region and endpoint settings, batch sizes, timeouts and retry values.</v>
+        <v>How one JAR serves several organizations and stores, and how the right configuration is selected at run time.</v>
       </c>
       <c r="E24" t="str">
         <v>Code walkthrough</v>
@@ -1337,16 +1337,16 @@
         <v/>
       </c>
       <c r="C25" t="str">
-        <v>Configuration per environment and per store</v>
+        <v>Mapping in the console versus mapping in the payload</v>
       </c>
       <c r="D25" t="str">
-        <v>How one JAR serves several organizations and stores, and how the right configuration is selected at run time.</v>
+        <v>Which values are set by the push payload, which by source mappings, and which wins.</v>
       </c>
       <c r="E25" t="str">
-        <v>Code walkthrough</v>
+        <v>Concept</v>
       </c>
       <c r="F25" t="str">
-        <v>Internal - config reference</v>
+        <v>docs.coveo.com - search: mapping rules</v>
       </c>
       <c r="G25" t="str">
         <v/>
@@ -1375,16 +1375,16 @@
         <v/>
       </c>
       <c r="C26" t="str">
-        <v>Mapping in the console versus mapping in the payload</v>
+        <v>Prove the wiring on non-prod before prod</v>
       </c>
       <c r="D26" t="str">
-        <v>Which values are set by the push payload, which by source mappings, and which wins.</v>
+        <v>A dry run that confirms key, source and mapping are correct without touching production content.</v>
       </c>
       <c r="E26" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F26" t="str">
-        <v>docs.coveo.com - search: mapping rules</v>
+        <v>Internal - runbook</v>
       </c>
       <c r="G26" t="str">
         <v/>
@@ -1407,22 +1407,22 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>3. Dashboard configuration to the indexing JAR</v>
+        <v>4. Indexing JAR, process and code walkthrough</v>
       </c>
       <c r="B27" t="str">
-        <v/>
+        <v>Read the JAR, run it against non-prod, and explain each stage of a run.</v>
       </c>
       <c r="C27" t="str">
-        <v>Prove the wiring on non-prod before prod</v>
+        <v>End-to-end shape of an indexing run</v>
       </c>
       <c r="D27" t="str">
-        <v>A dry run that confirms key, source and mapping are correct without touching production content.</v>
+        <v>Trigger, fetch from the source system, transform, push to Coveo, report. Where each step can stop.</v>
       </c>
       <c r="E27" t="str">
-        <v>Hands-on</v>
+        <v>Concept</v>
       </c>
       <c r="F27" t="str">
-        <v>Internal - runbook</v>
+        <v>Internal - architecture diagram</v>
       </c>
       <c r="G27" t="str">
         <v/>
@@ -1448,19 +1448,19 @@
         <v>4. Indexing JAR, process and code walkthrough</v>
       </c>
       <c r="B28" t="str">
-        <v>Read the JAR, run it against non-prod, and explain each stage of a run.</v>
+        <v/>
       </c>
       <c r="C28" t="str">
-        <v>End-to-end shape of an indexing run</v>
+        <v>Project layout and entry points</v>
       </c>
       <c r="D28" t="str">
-        <v>Trigger, fetch from the source system, transform, push to Coveo, report. Where each step can stop.</v>
+        <v>Modules, main class, how the JAR is built and versioned, and where to start reading.</v>
       </c>
       <c r="E28" t="str">
-        <v>Concept</v>
+        <v>Code walkthrough</v>
       </c>
       <c r="F28" t="str">
-        <v>Internal - architecture diagram</v>
+        <v>Internal - repository</v>
       </c>
       <c r="G28" t="str">
         <v/>
@@ -1489,16 +1489,16 @@
         <v/>
       </c>
       <c r="C29" t="str">
-        <v>Project layout and entry points</v>
+        <v>Data model and item identifiers</v>
       </c>
       <c r="D29" t="str">
-        <v>Modules, main class, how the JAR is built and versioned, and where to start reading.</v>
+        <v>The fields we send, how an item URI or permanent ID is composed, and why a stable identifier matters.</v>
       </c>
       <c r="E29" t="str">
         <v>Code walkthrough</v>
       </c>
       <c r="F29" t="str">
-        <v>Internal - repository</v>
+        <v>docs.coveo.com - search: item identifier</v>
       </c>
       <c r="G29" t="str">
         <v/>
@@ -1527,16 +1527,16 @@
         <v/>
       </c>
       <c r="C30" t="str">
-        <v>Data model and item identifiers</v>
+        <v>Batch push and Stream API</v>
       </c>
       <c r="D30" t="str">
-        <v>The fields we send, how an item URI or permanent ID is composed, and why a stable identifier matters.</v>
+        <v>Single item, batch and stream operations. Which the JAR uses for a delta run and which for a rebuild.</v>
       </c>
       <c r="E30" t="str">
         <v>Code walkthrough</v>
       </c>
       <c r="F30" t="str">
-        <v>docs.coveo.com - search: item identifier</v>
+        <v>docs.coveo.com - search: Stream API</v>
       </c>
       <c r="G30" t="str">
         <v/>
@@ -1565,16 +1565,16 @@
         <v/>
       </c>
       <c r="C31" t="str">
-        <v>Batch push and Stream API</v>
+        <v>Full rebuild, delta run and deletions</v>
       </c>
       <c r="D31" t="str">
-        <v>Single item, batch and stream operations. Which the JAR uses for a delta run and which for a rebuild.</v>
+        <v>How a full run differs from an incremental one, and how removals reach the index.</v>
       </c>
       <c r="E31" t="str">
-        <v>Code walkthrough</v>
+        <v>Concept</v>
       </c>
       <c r="F31" t="str">
-        <v>docs.coveo.com - search: Stream API</v>
+        <v>docs.coveo.com - search: delete items</v>
       </c>
       <c r="G31" t="str">
         <v/>
@@ -1603,16 +1603,16 @@
         <v/>
       </c>
       <c r="C32" t="str">
-        <v>Full rebuild, delta run and deletions</v>
+        <v>Scheduling, retries and idempotency</v>
       </c>
       <c r="D32" t="str">
-        <v>How a full run differs from an incremental one, and how removals reach the index.</v>
+        <v>How runs are scheduled, what happens on overlap, and why a rerun must be safe.</v>
       </c>
       <c r="E32" t="str">
-        <v>Concept</v>
+        <v>Code walkthrough</v>
       </c>
       <c r="F32" t="str">
-        <v>docs.coveo.com - search: delete items</v>
+        <v>Internal - repository</v>
       </c>
       <c r="G32" t="str">
         <v/>
@@ -1641,16 +1641,16 @@
         <v/>
       </c>
       <c r="C33" t="str">
-        <v>Scheduling, retries and idempotency</v>
+        <v>Logging, metrics and run records</v>
       </c>
       <c r="D33" t="str">
-        <v>How runs are scheduled, what happens on overlap, and why a rerun must be safe.</v>
+        <v>What the JAR logs, where the logs go, and what a healthy run looks like.</v>
       </c>
       <c r="E33" t="str">
         <v>Code walkthrough</v>
       </c>
       <c r="F33" t="str">
-        <v>Internal - repository</v>
+        <v>Internal - logging</v>
       </c>
       <c r="G33" t="str">
         <v/>
@@ -1679,19 +1679,19 @@
         <v/>
       </c>
       <c r="C34" t="str">
-        <v>Logging, metrics and run records</v>
+        <v>Run the JAR yourself against non-prod</v>
       </c>
       <c r="D34" t="str">
-        <v>What the JAR logs, where the logs go, and what a healthy run looks like.</v>
+        <v>Build, configure and execute a run, then confirm the result in the Content Browser.</v>
       </c>
       <c r="E34" t="str">
-        <v>Code walkthrough</v>
+        <v>Hands-on</v>
       </c>
       <c r="F34" t="str">
-        <v>Internal - logging</v>
+        <v>Internal - runbook</v>
       </c>
       <c r="G34" t="str">
-        <v/>
+        <v>The first real exit check for this stage.</v>
       </c>
       <c r="H34" t="str">
         <v>No</v>
@@ -1711,25 +1711,25 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>4. Indexing JAR, process and code walkthrough</v>
+        <v>5. Coveo APIs used by the JAR, and Swagger</v>
       </c>
       <c r="B35" t="str">
-        <v/>
+        <v>Call the Coveo APIs the JAR uses directly, and read the API reference unaided.</v>
       </c>
       <c r="C35" t="str">
-        <v>Run the JAR yourself against non-prod</v>
+        <v>Push API: add, update and delete</v>
       </c>
       <c r="D35" t="str">
-        <v>Build, configure and execute a run, then confirm the result in the Content Browser.</v>
+        <v>The endpoints the JAR calls, required headers, payload shape and expected responses.</v>
       </c>
       <c r="E35" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F35" t="str">
-        <v>Internal - runbook</v>
+        <v>docs.coveo.com - search: Push API</v>
       </c>
       <c r="G35" t="str">
-        <v>The first real exit check for this stage.</v>
+        <v/>
       </c>
       <c r="H35" t="str">
         <v>No</v>
@@ -1752,19 +1752,19 @@
         <v>5. Coveo APIs used by the JAR, and Swagger</v>
       </c>
       <c r="B36" t="str">
-        <v>Call the Coveo APIs the JAR uses directly, and read the API reference unaided.</v>
+        <v/>
       </c>
       <c r="C36" t="str">
-        <v>Push API: add, update and delete</v>
+        <v>Stream API: open, chunk, close</v>
       </c>
       <c r="D36" t="str">
-        <v>The endpoints the JAR calls, required headers, payload shape and expected responses.</v>
+        <v>When a stream is the right choice and what happens if a stream is left open.</v>
       </c>
       <c r="E36" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F36" t="str">
-        <v>docs.coveo.com - search: Push API</v>
+        <v>docs.coveo.com - search: Stream API</v>
       </c>
       <c r="G36" t="str">
         <v/>
@@ -1793,16 +1793,16 @@
         <v/>
       </c>
       <c r="C37" t="str">
-        <v>Stream API: open, chunk, close</v>
+        <v>Source status and activity endpoints</v>
       </c>
       <c r="D37" t="str">
-        <v>When a stream is the right choice and what happens if a stream is left open.</v>
+        <v>Setting source status, reading activity, and using it to confirm a run landed.</v>
       </c>
       <c r="E37" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F37" t="str">
-        <v>docs.coveo.com - search: Stream API</v>
+        <v>docs.coveo.com - search: source status</v>
       </c>
       <c r="G37" t="str">
         <v/>
@@ -1831,16 +1831,16 @@
         <v/>
       </c>
       <c r="C38" t="str">
-        <v>Source status and activity endpoints</v>
+        <v>Fields and mappings management APIs</v>
       </c>
       <c r="D38" t="str">
-        <v>Setting source status, reading activity, and using it to confirm a run landed.</v>
+        <v>Creating and editing fields and mappings through the API rather than the console.</v>
       </c>
       <c r="E38" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F38" t="str">
-        <v>docs.coveo.com - search: source status</v>
+        <v>docs.coveo.com - search: fields API</v>
       </c>
       <c r="G38" t="str">
         <v/>
@@ -1869,16 +1869,16 @@
         <v/>
       </c>
       <c r="C39" t="str">
-        <v>Fields and mappings management APIs</v>
+        <v>Swagger and the API reference walkthrough</v>
       </c>
       <c r="D39" t="str">
-        <v>Creating and editing fields and mappings through the API rather than the console.</v>
+        <v>Authenticating in the reference, running a call, reading request and response models.</v>
       </c>
       <c r="E39" t="str">
-        <v>Hands-on</v>
+        <v>Demo</v>
       </c>
       <c r="F39" t="str">
-        <v>docs.coveo.com - search: fields API</v>
+        <v>docs.coveo.com - search: API reference</v>
       </c>
       <c r="G39" t="str">
         <v/>
@@ -1907,16 +1907,16 @@
         <v/>
       </c>
       <c r="C40" t="str">
-        <v>Swagger and the API reference walkthrough</v>
+        <v>Limits and error codes</v>
       </c>
       <c r="D40" t="str">
-        <v>Authenticating in the reference, running a call, reading request and response models.</v>
+        <v>Rate limits, payload size limits, and what each HTTP status from Coveo actually means for a run.</v>
       </c>
       <c r="E40" t="str">
-        <v>Demo</v>
+        <v>Concept</v>
       </c>
       <c r="F40" t="str">
-        <v>docs.coveo.com - search: API reference</v>
+        <v>docs.coveo.com - search: API error codes</v>
       </c>
       <c r="G40" t="str">
         <v/>
@@ -1939,22 +1939,22 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>5. Coveo APIs used by the JAR, and Swagger</v>
+        <v>6. Indexing failure debug and config validation</v>
       </c>
       <c r="B41" t="str">
-        <v/>
+        <v>Take a failed indexing run and get to the cause without escalating.</v>
       </c>
       <c r="C41" t="str">
-        <v>Limits and error codes</v>
+        <v>Read a failed run: JAR log and Coveo activity</v>
       </c>
       <c r="D41" t="str">
-        <v>Rate limits, payload size limits, and what each HTTP status from Coveo actually means for a run.</v>
+        <v>Line up the JAR's own error with the source activity entry in the console.</v>
       </c>
       <c r="E41" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F41" t="str">
-        <v>docs.coveo.com - search: API error codes</v>
+        <v>docs.coveo.com - search: source activity</v>
       </c>
       <c r="G41" t="str">
         <v/>
@@ -1980,19 +1980,19 @@
         <v>6. Indexing failure debug and config validation</v>
       </c>
       <c r="B42" t="str">
-        <v>Take a failed indexing run and get to the cause without escalating.</v>
+        <v/>
       </c>
       <c r="C42" t="str">
-        <v>Read a failed run: JAR log and Coveo activity</v>
+        <v>Confirm an item in the Content Browser</v>
       </c>
       <c r="D42" t="str">
-        <v>Line up the JAR's own error with the source activity entry in the console.</v>
+        <v>Check that an item exists, and inspect its fields and permissions.</v>
       </c>
       <c r="E42" t="str">
-        <v>Hands-on</v>
+        <v>Demo</v>
       </c>
       <c r="F42" t="str">
-        <v>docs.coveo.com - search: source activity</v>
+        <v>docs.coveo.com - search: Content Browser</v>
       </c>
       <c r="G42" t="str">
         <v/>
@@ -2021,16 +2021,16 @@
         <v/>
       </c>
       <c r="C43" t="str">
-        <v>Confirm an item in the Content Browser</v>
+        <v>The failures we actually see</v>
       </c>
       <c r="D43" t="str">
-        <v>Check that an item exists, and inspect its fields and permissions.</v>
+        <v>Bad or missing mapping, missing field, expired or under-privileged key, payload too large, malformed JSON, source in the wrong state.</v>
       </c>
       <c r="E43" t="str">
-        <v>Demo</v>
+        <v>Concept</v>
       </c>
       <c r="F43" t="str">
-        <v>docs.coveo.com - search: Content Browser</v>
+        <v>Internal - incident history</v>
       </c>
       <c r="G43" t="str">
         <v/>
@@ -2059,16 +2059,16 @@
         <v/>
       </c>
       <c r="C44" t="str">
-        <v>The failures we actually see</v>
+        <v>Item-level error versus rejected batch</v>
       </c>
       <c r="D44" t="str">
-        <v>Bad or missing mapping, missing field, expired or under-privileged key, payload too large, malformed JSON, source in the wrong state.</v>
+        <v>Telling a single bad item apart from a whole batch that never landed, and what each needs.</v>
       </c>
       <c r="E44" t="str">
         <v>Concept</v>
       </c>
       <c r="F44" t="str">
-        <v>Internal - incident history</v>
+        <v>docs.coveo.com - search: push error</v>
       </c>
       <c r="G44" t="str">
         <v/>
@@ -2097,16 +2097,16 @@
         <v/>
       </c>
       <c r="C45" t="str">
-        <v>Item-level error versus rejected batch</v>
+        <v>Configuration validation checklist</v>
       </c>
       <c r="D45" t="str">
-        <v>Telling a single bad item apart from a whole batch that never landed, and what each needs.</v>
+        <v>What to re-check after any configuration change, in order, before declaring a run healthy.</v>
       </c>
       <c r="E45" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F45" t="str">
-        <v>docs.coveo.com - search: push error</v>
+        <v>Internal - runbook</v>
       </c>
       <c r="G45" t="str">
         <v/>
@@ -2135,10 +2135,10 @@
         <v/>
       </c>
       <c r="C46" t="str">
-        <v>Configuration validation checklist</v>
+        <v>Re-drive a failed batch safely</v>
       </c>
       <c r="D46" t="str">
-        <v>What to re-check after any configuration change, in order, before declaring a run healthy.</v>
+        <v>Replaying without duplicating items or wiping good content.</v>
       </c>
       <c r="E46" t="str">
         <v>Hands-on</v>
@@ -2173,16 +2173,16 @@
         <v/>
       </c>
       <c r="C47" t="str">
-        <v>Re-drive a failed batch safely</v>
+        <v>Rebuild, refresh and rescan</v>
       </c>
       <c r="D47" t="str">
-        <v>Replaying without duplicating items or wiping good content.</v>
+        <v>What each does, what it costs, and how to choose under time pressure.</v>
       </c>
       <c r="E47" t="str">
-        <v>Hands-on</v>
+        <v>Concept</v>
       </c>
       <c r="F47" t="str">
-        <v>Internal - runbook</v>
+        <v>docs.coveo.com - search: refresh rescan rebuild</v>
       </c>
       <c r="G47" t="str">
         <v/>
@@ -2205,22 +2205,22 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>6. Indexing failure debug and config validation</v>
+        <v>7. Store go-live validation and keys</v>
       </c>
       <c r="B48" t="str">
-        <v/>
+        <v>Validate and cut over a new store on your own, with a rollback ready.</v>
       </c>
       <c r="C48" t="str">
-        <v>Rebuild, refresh and rescan</v>
+        <v>Go-live checklist for a new store</v>
       </c>
       <c r="D48" t="str">
-        <v>What each does, what it costs, and how to choose under time pressure.</v>
+        <v>Every configuration item and key needed before a store can serve traffic.</v>
       </c>
       <c r="E48" t="str">
         <v>Concept</v>
       </c>
       <c r="F48" t="str">
-        <v>docs.coveo.com - search: refresh rescan rebuild</v>
+        <v>Internal - go-live checklist</v>
       </c>
       <c r="G48" t="str">
         <v/>
@@ -2246,19 +2246,19 @@
         <v>7. Store go-live validation and keys</v>
       </c>
       <c r="B49" t="str">
-        <v>Validate and cut over a new store on your own, with a rollback ready.</v>
+        <v/>
       </c>
       <c r="C49" t="str">
-        <v>Go-live checklist for a new store</v>
+        <v>Store configuration: catalog, source, pipeline, search hub, fields</v>
       </c>
       <c r="D49" t="str">
-        <v>Every configuration item and key needed before a store can serve traffic.</v>
+        <v>What is created per store, what is shared, and the naming we follow.</v>
       </c>
       <c r="E49" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F49" t="str">
-        <v>Internal - go-live checklist</v>
+        <v>docs.coveo.com - search: search hub</v>
       </c>
       <c r="G49" t="str">
         <v/>
@@ -2287,19 +2287,19 @@
         <v/>
       </c>
       <c r="C50" t="str">
-        <v>Store configuration: catalog, source, pipeline, search hub, fields</v>
+        <v>Keys and access for the new environment</v>
       </c>
       <c r="D50" t="str">
-        <v>What is created per store, what is shared, and the naming we follow.</v>
+        <v>Requesting keys, confirming privileges, and recording them in the secret store.</v>
       </c>
       <c r="E50" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F50" t="str">
-        <v>docs.coveo.com - search: search hub</v>
+        <v>Internal - secret management</v>
       </c>
       <c r="G50" t="str">
-        <v/>
+        <v>Values go in the secret store only.</v>
       </c>
       <c r="H50" t="str">
         <v>No</v>
@@ -2325,19 +2325,19 @@
         <v/>
       </c>
       <c r="C51" t="str">
-        <v>Keys and access for the new environment</v>
+        <v>Non-prod parity check</v>
       </c>
       <c r="D51" t="str">
-        <v>Requesting keys, confirming privileges, and recording them in the secret store.</v>
+        <v>Proving non-prod and prod configuration match before cutover.</v>
       </c>
       <c r="E51" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F51" t="str">
-        <v>Internal - secret management</v>
+        <v>Internal - runbook</v>
       </c>
       <c r="G51" t="str">
-        <v>Values go in the secret store only.</v>
+        <v/>
       </c>
       <c r="H51" t="str">
         <v>No</v>
@@ -2363,16 +2363,16 @@
         <v/>
       </c>
       <c r="C52" t="str">
-        <v>Non-prod parity check</v>
+        <v>Cutover sequence and rollback</v>
       </c>
       <c r="D52" t="str">
-        <v>Proving non-prod and prod configuration match before cutover.</v>
+        <v>Order of operations on go-live day, who signs off, and how we roll back.</v>
       </c>
       <c r="E52" t="str">
-        <v>Hands-on</v>
+        <v>Shadowing</v>
       </c>
       <c r="F52" t="str">
-        <v>Internal - runbook</v>
+        <v>Internal - go-live plan</v>
       </c>
       <c r="G52" t="str">
         <v/>
@@ -2401,16 +2401,16 @@
         <v/>
       </c>
       <c r="C53" t="str">
-        <v>Cutover sequence and rollback</v>
+        <v>Post-go-live smoke checks</v>
       </c>
       <c r="D53" t="str">
-        <v>Order of operations on go-live day, who signs off, and how we roll back.</v>
+        <v>Indexed counts, sample queries, facets, and analytics events arriving.</v>
       </c>
       <c r="E53" t="str">
-        <v>Shadowing</v>
+        <v>Hands-on</v>
       </c>
       <c r="F53" t="str">
-        <v>Internal - go-live plan</v>
+        <v>Internal - runbook</v>
       </c>
       <c r="G53" t="str">
         <v/>
@@ -2433,22 +2433,22 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>7. Store go-live validation and keys</v>
+        <v>8. Response inspector, analytics and user journey</v>
       </c>
       <c r="B54" t="str">
-        <v/>
+        <v>Follow one user journey from the search response through to the analytics record.</v>
       </c>
       <c r="C54" t="str">
-        <v>Post-go-live smoke checks</v>
+        <v>Read a search response</v>
       </c>
       <c r="D54" t="str">
-        <v>Indexed counts, sample queries, facets, and analytics events arriving.</v>
+        <v>Response structure, returned fields, ranking information, and total counts.</v>
       </c>
       <c r="E54" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F54" t="str">
-        <v>Internal - runbook</v>
+        <v>docs.coveo.com - search: Search API response</v>
       </c>
       <c r="G54" t="str">
         <v/>
@@ -2474,19 +2474,19 @@
         <v>8. Response inspector, analytics and user journey</v>
       </c>
       <c r="B55" t="str">
-        <v>Follow one user journey from the search response through to the analytics record.</v>
+        <v/>
       </c>
       <c r="C55" t="str">
-        <v>Read a search response</v>
+        <v>Debug mode and the execution report</v>
       </c>
       <c r="D55" t="str">
-        <v>Response structure, returned fields, ranking information, and total counts.</v>
+        <v>Appending debug to a query and reading the execution report to see what the pipeline did.</v>
       </c>
       <c r="E55" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F55" t="str">
-        <v>docs.coveo.com - search: Search API response</v>
+        <v>docs.coveo.com - search: execution report</v>
       </c>
       <c r="G55" t="str">
         <v/>
@@ -2515,16 +2515,16 @@
         <v/>
       </c>
       <c r="C56" t="str">
-        <v>Debug mode and the execution report</v>
+        <v>Relevance inspector</v>
       </c>
       <c r="D56" t="str">
-        <v>Appending debug to a query and reading the execution report to see what the pipeline did.</v>
+        <v>Opening the inspector, reading ranking contributions, and spotting an over-boosted pipeline.</v>
       </c>
       <c r="E56" t="str">
-        <v>Hands-on</v>
+        <v>Demo</v>
       </c>
       <c r="F56" t="str">
-        <v>docs.coveo.com - search: execution report</v>
+        <v>docs.coveo.com - search: relevance inspector</v>
       </c>
       <c r="G56" t="str">
         <v/>
@@ -2553,16 +2553,16 @@
         <v/>
       </c>
       <c r="C57" t="str">
-        <v>Relevance inspector</v>
+        <v>Analytics event types</v>
       </c>
       <c r="D57" t="str">
-        <v>Opening the inspector, reading ranking contributions, and spotting an over-boosted pipeline.</v>
+        <v>Search, click, custom, view and commerce events, and which of them we depend on.</v>
       </c>
       <c r="E57" t="str">
-        <v>Demo</v>
+        <v>Concept</v>
       </c>
       <c r="F57" t="str">
-        <v>docs.coveo.com - search: relevance inspector</v>
+        <v>docs.coveo.com - search: usage analytics events</v>
       </c>
       <c r="G57" t="str">
         <v/>
@@ -2591,16 +2591,16 @@
         <v/>
       </c>
       <c r="C58" t="str">
-        <v>Analytics event types</v>
+        <v>How events reach Coveo</v>
       </c>
       <c r="D58" t="str">
-        <v>Search, click, custom, view and commerce events, and which of them we depend on.</v>
+        <v>What the front end sends, what we send server-side, and the fields that must be present.</v>
       </c>
       <c r="E58" t="str">
         <v>Concept</v>
       </c>
       <c r="F58" t="str">
-        <v>docs.coveo.com - search: usage analytics events</v>
+        <v>docs.coveo.com - search: send analytics events</v>
       </c>
       <c r="G58" t="str">
         <v/>
@@ -2629,16 +2629,16 @@
         <v/>
       </c>
       <c r="C59" t="str">
-        <v>How events reach Coveo</v>
+        <v>Follow one visit end to end</v>
       </c>
       <c r="D59" t="str">
-        <v>What the front end sends, what we send server-side, and the fields that must be present.</v>
+        <v>Take a single visit and trace query, results, clicks and conversion.</v>
       </c>
       <c r="E59" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F59" t="str">
-        <v>docs.coveo.com - search: send analytics events</v>
+        <v>docs.coveo.com - search: visit browser</v>
       </c>
       <c r="G59" t="str">
         <v/>
@@ -2667,19 +2667,19 @@
         <v/>
       </c>
       <c r="C60" t="str">
-        <v>Follow one visit end to end</v>
+        <v>Event data quality</v>
       </c>
       <c r="D60" t="str">
-        <v>Take a single visit and trace query, results, clicks and conversion.</v>
+        <v>Missing, duplicated or mistyped events, how we detect them, and what they break downstream.</v>
       </c>
       <c r="E60" t="str">
-        <v>Hands-on</v>
+        <v>Concept</v>
       </c>
       <c r="F60" t="str">
-        <v>docs.coveo.com - search: visit browser</v>
+        <v>docs.coveo.com - search: analytics data health</v>
       </c>
       <c r="G60" t="str">
-        <v/>
+        <v>Bad events quietly degrade every model.</v>
       </c>
       <c r="H60" t="str">
         <v>No</v>
@@ -2699,25 +2699,25 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>8. Response inspector, analytics and user journey</v>
+        <v>9. Merchandising Hub rules and configuration</v>
       </c>
       <c r="B61" t="str">
-        <v/>
+        <v>Support merchandising rules and explain why a rule did or didn't take effect.</v>
       </c>
       <c r="C61" t="str">
-        <v>Event data quality</v>
+        <v>What the Merchandising Hub is and who uses it</v>
       </c>
       <c r="D61" t="str">
-        <v>Missing, duplicated or mistyped events, how we detect them, and what they break downstream.</v>
+        <v>The split between business-owned merchandising and our configuration.</v>
       </c>
       <c r="E61" t="str">
         <v>Concept</v>
       </c>
       <c r="F61" t="str">
-        <v>docs.coveo.com - search: analytics data health</v>
+        <v>docs.coveo.com - search: Merchandising Hub</v>
       </c>
       <c r="G61" t="str">
-        <v>Bad events quietly degrade every model.</v>
+        <v/>
       </c>
       <c r="H61" t="str">
         <v>No</v>
@@ -2740,19 +2740,19 @@
         <v>9. Merchandising Hub rules and configuration</v>
       </c>
       <c r="B62" t="str">
-        <v>Support merchandising rules and explain why a rule did or didn't take effect.</v>
+        <v/>
       </c>
       <c r="C62" t="str">
-        <v>What the Merchandising Hub is and who uses it</v>
+        <v>Product listings and catalog configuration behind it</v>
       </c>
       <c r="D62" t="str">
-        <v>The split between business-owned merchandising and our configuration.</v>
+        <v>Catalog structure, product grouping and availability, and what the hub relies on from the index.</v>
       </c>
       <c r="E62" t="str">
         <v>Concept</v>
       </c>
       <c r="F62" t="str">
-        <v>docs.coveo.com - search: Merchandising Hub</v>
+        <v>docs.coveo.com - search: product listing configuration</v>
       </c>
       <c r="G62" t="str">
         <v/>
@@ -2781,16 +2781,16 @@
         <v/>
       </c>
       <c r="C63" t="str">
-        <v>Product listings and catalog configuration behind it</v>
+        <v>Rule types and what each one does</v>
       </c>
       <c r="D63" t="str">
-        <v>Catalog structure, product grouping and availability, and what the hub relies on from the index.</v>
+        <v>Boost, bury, pin, block and filter rules, and their order of effect.</v>
       </c>
       <c r="E63" t="str">
-        <v>Concept</v>
+        <v>Demo</v>
       </c>
       <c r="F63" t="str">
-        <v>docs.coveo.com - search: product listing configuration</v>
+        <v>docs.coveo.com - search: merchandising rules</v>
       </c>
       <c r="G63" t="str">
         <v/>
@@ -2819,16 +2819,16 @@
         <v/>
       </c>
       <c r="C64" t="str">
-        <v>Rule types and what each one does</v>
+        <v>Merchandising rules versus query pipeline statements</v>
       </c>
       <c r="D64" t="str">
-        <v>Boost, bury, pin, block and filter rules, and their order of effect.</v>
+        <v>Which layer to use for which requirement, and how they interact.</v>
       </c>
       <c r="E64" t="str">
-        <v>Demo</v>
+        <v>Concept</v>
       </c>
       <c r="F64" t="str">
-        <v>docs.coveo.com - search: merchandising rules</v>
+        <v>docs.coveo.com - search: ranking rules</v>
       </c>
       <c r="G64" t="str">
         <v/>
@@ -2857,16 +2857,16 @@
         <v/>
       </c>
       <c r="C65" t="str">
-        <v>Merchandising rules versus query pipeline statements</v>
+        <v>Index-side requirements for merchandising</v>
       </c>
       <c r="D65" t="str">
-        <v>Which layer to use for which requirement, and how they interact.</v>
+        <v>Fields, availability data and grouping that must be indexed correctly for rules to work.</v>
       </c>
       <c r="E65" t="str">
         <v>Concept</v>
       </c>
       <c r="F65" t="str">
-        <v>docs.coveo.com - search: ranking rules</v>
+        <v>docs.coveo.com - search: catalog fields</v>
       </c>
       <c r="G65" t="str">
         <v/>
@@ -2895,16 +2895,16 @@
         <v/>
       </c>
       <c r="C66" t="str">
-        <v>Index-side requirements for merchandising</v>
+        <v>Troubleshoot a rule that has no effect</v>
       </c>
       <c r="D66" t="str">
-        <v>Fields, availability data and grouping that must be indexed correctly for rules to work.</v>
+        <v>Check the listing, the condition, the pipeline, then the underlying data.</v>
       </c>
       <c r="E66" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F66" t="str">
-        <v>docs.coveo.com - search: catalog fields</v>
+        <v>Internal - incident history</v>
       </c>
       <c r="G66" t="str">
         <v/>
@@ -2933,16 +2933,16 @@
         <v/>
       </c>
       <c r="C67" t="str">
-        <v>Troubleshoot a rule that has no effect</v>
+        <v>Change control for merchandising</v>
       </c>
       <c r="D67" t="str">
-        <v>Check the listing, the condition, the pipeline, then the underlying data.</v>
+        <v>Who approves, where changes are recorded, and how a rule is reverted.</v>
       </c>
       <c r="E67" t="str">
-        <v>Hands-on</v>
+        <v>Concept</v>
       </c>
       <c r="F67" t="str">
-        <v>Internal - incident history</v>
+        <v>Internal - ways of working</v>
       </c>
       <c r="G67" t="str">
         <v/>
@@ -2965,22 +2965,22 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>9. Merchandising Hub rules and configuration</v>
+        <v>10. Coveo models walkthrough and configuration</v>
       </c>
       <c r="B68" t="str">
-        <v/>
+        <v>Know which model solves which problem, what data it needs, and how it is wired to a pipeline.</v>
       </c>
       <c r="C68" t="str">
-        <v>Change control for merchandising</v>
+        <v>The model catalogue</v>
       </c>
       <c r="D68" t="str">
-        <v>Who approves, where changes are recorded, and how a rule is reverted.</v>
+        <v>ART, Query Suggestions and Predictive QS, DNE, Content Recommendations, Product Recommendations and IAPR, Smart Snippets, Relevance Generative Answering with its Semantic Encoder, Case Classification.</v>
       </c>
       <c r="E68" t="str">
         <v>Concept</v>
       </c>
       <c r="F68" t="str">
-        <v>Internal - ways of working</v>
+        <v>docs.coveo.com - search: Coveo Machine Learning models</v>
       </c>
       <c r="G68" t="str">
         <v/>
@@ -3006,19 +3006,19 @@
         <v>10. Coveo models walkthrough and configuration</v>
       </c>
       <c r="B69" t="str">
-        <v>Know which model solves which problem, what data it needs, and how it is wired to a pipeline.</v>
+        <v/>
       </c>
       <c r="C69" t="str">
-        <v>The model catalogue</v>
+        <v>What each model needs before it can work</v>
       </c>
       <c r="D69" t="str">
-        <v>ART, Query Suggestions and Predictive QS, DNE, Content Recommendations, Product Recommendations and IAPR, Smart Snippets, Relevance Generative Answering with its Semantic Encoder, Case Classification.</v>
+        <v>Event volume, content scope and field requirements. Why a model can sit idle.</v>
       </c>
       <c r="E69" t="str">
         <v>Concept</v>
       </c>
       <c r="F69" t="str">
-        <v>docs.coveo.com - search: Coveo Machine Learning models</v>
+        <v>docs.coveo.com - search: model requirements</v>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -3047,16 +3047,16 @@
         <v/>
       </c>
       <c r="C70" t="str">
-        <v>What each model needs before it can work</v>
+        <v>Create a model and associate it with a pipeline</v>
       </c>
       <c r="D70" t="str">
-        <v>Event volume, content scope and field requirements. Why a model can sit idle.</v>
+        <v>Configuration options, conditions, association order, and what order means at query time.</v>
       </c>
       <c r="E70" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F70" t="str">
-        <v>docs.coveo.com - search: model requirements</v>
+        <v>docs.coveo.com - search: model associations</v>
       </c>
       <c r="G70" t="str">
         <v/>
@@ -3085,16 +3085,16 @@
         <v/>
       </c>
       <c r="C71" t="str">
-        <v>Create a model and associate it with a pipeline</v>
+        <v>Commerce model specifics</v>
       </c>
       <c r="D71" t="str">
-        <v>Configuration options, conditions, association order, and what order means at query time.</v>
+        <v>Product recommendations and intent-aware ranking, and the catalog data they depend on.</v>
       </c>
       <c r="E71" t="str">
-        <v>Hands-on</v>
+        <v>Concept</v>
       </c>
       <c r="F71" t="str">
-        <v>docs.coveo.com - search: model associations</v>
+        <v>docs.coveo.com - search: Product Recommendations</v>
       </c>
       <c r="G71" t="str">
         <v/>
@@ -3123,16 +3123,16 @@
         <v/>
       </c>
       <c r="C72" t="str">
-        <v>Commerce model specifics</v>
+        <v>Training schedule, status and candidate review</v>
       </c>
       <c r="D72" t="str">
-        <v>Product recommendations and intent-aware ranking, and the catalog data they depend on.</v>
+        <v>When models retrain, how to read status, and how to review what a model would suggest.</v>
       </c>
       <c r="E72" t="str">
-        <v>Concept</v>
+        <v>Demo</v>
       </c>
       <c r="F72" t="str">
-        <v>docs.coveo.com - search: Product Recommendations</v>
+        <v>docs.coveo.com - search: review model information</v>
       </c>
       <c r="G72" t="str">
         <v/>
@@ -3161,16 +3161,16 @@
         <v/>
       </c>
       <c r="C73" t="str">
-        <v>Training schedule, status and candidate review</v>
+        <v>A/B testing a pipeline change</v>
       </c>
       <c r="D73" t="str">
-        <v>When models retrain, how to read status, and how to review what a model would suggest.</v>
+        <v>Setting up a split, choosing the metric, and how long to leave it running.</v>
       </c>
       <c r="E73" t="str">
-        <v>Demo</v>
+        <v>Concept</v>
       </c>
       <c r="F73" t="str">
-        <v>docs.coveo.com - search: review model information</v>
+        <v>docs.coveo.com - search: A/B test</v>
       </c>
       <c r="G73" t="str">
         <v/>
@@ -3199,16 +3199,16 @@
         <v/>
       </c>
       <c r="C74" t="str">
-        <v>A/B testing a pipeline change</v>
+        <v>What silently breaks a model</v>
       </c>
       <c r="D74" t="str">
-        <v>Setting up a split, choosing the metric, and how long to leave it running.</v>
+        <v>Event gaps, renamed fields, changed permissions, reindexing without care.</v>
       </c>
       <c r="E74" t="str">
         <v>Concept</v>
       </c>
       <c r="F74" t="str">
-        <v>docs.coveo.com - search: A/B test</v>
+        <v>Internal - incident history</v>
       </c>
       <c r="G74" t="str">
         <v/>
@@ -3231,22 +3231,22 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>10. Coveo models walkthrough and configuration</v>
+        <v>11. Configuration and useful APIs after go-live</v>
       </c>
       <c r="B75" t="str">
-        <v/>
+        <v>Run and audit the configuration day to day, and know when to escalate.</v>
       </c>
       <c r="C75" t="str">
-        <v>What silently breaks a model</v>
+        <v>Routine health checks</v>
       </c>
       <c r="D75" t="str">
-        <v>Event gaps, renamed fields, changed permissions, reindexing without care.</v>
+        <v>Source health, indexed counts, failed runs, quota and consumption. What we check and how often.</v>
       </c>
       <c r="E75" t="str">
-        <v>Concept</v>
+        <v>Hands-on</v>
       </c>
       <c r="F75" t="str">
-        <v>Internal - incident history</v>
+        <v>Internal - runbook</v>
       </c>
       <c r="G75" t="str">
         <v/>
@@ -3272,19 +3272,19 @@
         <v>11. Configuration and useful APIs after go-live</v>
       </c>
       <c r="B76" t="str">
-        <v>Run and audit the configuration day to day, and know when to escalate.</v>
+        <v/>
       </c>
       <c r="C76" t="str">
-        <v>Routine health checks</v>
+        <v>Resource snapshots and promoting configuration</v>
       </c>
       <c r="D76" t="str">
-        <v>Source health, indexed counts, failed runs, quota and consumption. What we check and how often.</v>
+        <v>Capturing configuration, comparing organizations, and applying a snapshot.</v>
       </c>
       <c r="E76" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F76" t="str">
-        <v>Internal - runbook</v>
+        <v>docs.coveo.com - search: resource snapshots</v>
       </c>
       <c r="G76" t="str">
         <v/>
@@ -3313,16 +3313,16 @@
         <v/>
       </c>
       <c r="C77" t="str">
-        <v>Resource snapshots and promoting configuration</v>
+        <v>Admin and Search APIs worth knowing</v>
       </c>
       <c r="D77" t="str">
-        <v>Capturing configuration, comparing organizations, and applying a snapshot.</v>
+        <v>Endpoints we use for reporting, audits and bulk checks after go-live.</v>
       </c>
       <c r="E77" t="str">
         <v>Hands-on</v>
       </c>
       <c r="F77" t="str">
-        <v>docs.coveo.com - search: resource snapshots</v>
+        <v>docs.coveo.com - search: platform API</v>
       </c>
       <c r="G77" t="str">
         <v/>
@@ -3351,16 +3351,16 @@
         <v/>
       </c>
       <c r="C78" t="str">
-        <v>Admin and Search APIs worth knowing</v>
+        <v>Monitoring and alerting</v>
       </c>
       <c r="D78" t="str">
-        <v>Endpoints we use for reporting, audits and bulk checks after go-live.</v>
+        <v>What is monitored today, what triggers an alert, and who receives it.</v>
       </c>
       <c r="E78" t="str">
-        <v>Hands-on</v>
+        <v>Concept</v>
       </c>
       <c r="F78" t="str">
-        <v>docs.coveo.com - search: platform API</v>
+        <v>Internal - monitoring</v>
       </c>
       <c r="G78" t="str">
         <v/>
@@ -3389,16 +3389,16 @@
         <v/>
       </c>
       <c r="C79" t="str">
-        <v>Monitoring and alerting</v>
+        <v>Support and escalation</v>
       </c>
       <c r="D79" t="str">
-        <v>What is monitored today, what triggers an alert, and who receives it.</v>
+        <v>Coveo support channels, what a useful ticket contains, and our internal escalation path.</v>
       </c>
       <c r="E79" t="str">
         <v>Concept</v>
       </c>
       <c r="F79" t="str">
-        <v>Internal - monitoring</v>
+        <v>Internal - escalation matrix</v>
       </c>
       <c r="G79" t="str">
         <v/>
@@ -3427,16 +3427,16 @@
         <v/>
       </c>
       <c r="C80" t="str">
-        <v>Support and escalation</v>
+        <v>Documentation and ownership handover</v>
       </c>
       <c r="D80" t="str">
-        <v>Coveo support channels, what a useful ticket contains, and our internal escalation path.</v>
+        <v>What you own from here, where the runbook lives, and what you keep current.</v>
       </c>
       <c r="E80" t="str">
-        <v>Concept</v>
+        <v>Reading</v>
       </c>
       <c r="F80" t="str">
-        <v>Internal - escalation matrix</v>
+        <v>Internal - runbook</v>
       </c>
       <c r="G80" t="str">
         <v/>
@@ -3465,19 +3465,19 @@
         <v/>
       </c>
       <c r="C81" t="str">
-        <v>Documentation and ownership handover</v>
+        <v>Lead one indexing change end to end</v>
       </c>
       <c r="D81" t="str">
-        <v>What you own from here, where the runbook lives, and what you keep current.</v>
+        <v>Plan it, validate on non-prod, apply to prod and report it, with me only observing.</v>
       </c>
       <c r="E81" t="str">
-        <v>Reading</v>
+        <v>Shadowing</v>
       </c>
       <c r="F81" t="str">
-        <v>Internal - runbook</v>
+        <v>Internal</v>
       </c>
       <c r="G81" t="str">
-        <v/>
+        <v>The real exit criterion for this roadmap.</v>
       </c>
       <c r="H81" t="str">
         <v>No</v>
@@ -3492,50 +3492,12 @@
         <v/>
       </c>
       <c r="L81" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="str">
-        <v>11. Configuration and useful APIs after go-live</v>
-      </c>
-      <c r="B82" t="str">
-        <v/>
-      </c>
-      <c r="C82" t="str">
-        <v>Lead one indexing change end to end</v>
-      </c>
-      <c r="D82" t="str">
-        <v>Plan it, validate on non-prod, apply to prod and report it, with me only observing.</v>
-      </c>
-      <c r="E82" t="str">
-        <v>Shadowing</v>
-      </c>
-      <c r="F82" t="str">
-        <v>Internal</v>
-      </c>
-      <c r="G82" t="str">
-        <v>The real exit criterion for this roadmap.</v>
-      </c>
-      <c r="H82" t="str">
-        <v>No</v>
-      </c>
-      <c r="I82" t="str">
-        <v/>
-      </c>
-      <c r="J82" t="str">
-        <v>Not started</v>
-      </c>
-      <c r="K82" t="str">
-        <v/>
-      </c>
-      <c r="L82" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L81"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
KT progress: names set by Akshay
</commit_message>
<xml_diff>
--- a/coveo-kt-tracker.xlsx
+++ b/coveo-kt-tracker.xlsx
@@ -3184,7 +3184,7 @@
         <v>Explaining</v>
       </c>
       <c r="B2" t="str">
-        <v>AKSHAY</v>
+        <v>Akshay</v>
       </c>
     </row>
     <row r="3">
@@ -3192,7 +3192,7 @@
         <v>Learning</v>
       </c>
       <c r="B3" t="str">
-        <v>DIVYASHREE</v>
+        <v>Divyashree</v>
       </c>
     </row>
   </sheetData>

</xml_diff>